<commit_message>
feat: implement comprehensive Notion integration for job syncing, metadata management, and AI analysis reporting
</commit_message>
<xml_diff>
--- a/reports/jobs_report_2026-08-05.xlsx
+++ b/reports/jobs_report_2026-08-05.xlsx
@@ -488,22 +488,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -554,20 +556,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Data Extração</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Link de Candidatura</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Estado Candidatura</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Análise da IA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notas Pessoais</t>
         </is>
@@ -575,7 +587,7 @@
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>85</v>
+        <v>82.5</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -584,7 +596,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Neotalent Conclusion</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -609,7 +621,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Junior / Entry Level</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -619,29 +631,327 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
           <t>ITJobs.pt</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, foco em IA e tecnologia</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>DATA SCIENCE CONSULTANT LISBON</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Management Solutions</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Lisboa, Lisbon, Portugal</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Presencial / Híbrido</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Não especificado</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>python, machine learning, monte carlo</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Recém-licenciado</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05 23:30:36</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, habilidades relevantes</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>BI Machine Learning BI/26_016_ConvergeAI_EPMQ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Associação CCG - Centro de Computação Gráfica</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Presencial / Híbrido</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Não especificado</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>python, fastapi, llm, machine learning</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Recém-licenciado</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Net-Empregos</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de Machine Learning e BI</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>BI Data Scientist</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>PrimeIT</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Lisbon, Portugal</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Presencial / Híbrido</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Não especificado</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>sql, git, llm</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Recém-licenciado</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05 23:30:37</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Habilidades em BI e data science relevantes</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>BJAK</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Presencial / Híbrido</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Não especificado</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>python, rag, llm</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Recém-licenciado</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05 23:30:15</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, oportunidade de trabalhar em AI-native systems</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="L2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Por Candidatar,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
+    <dataValidation sqref="M2:M6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por Candidatar,Candidatura feita,Cadidatura feita,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -653,22 +963,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -719,20 +1031,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Data Extração</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Link de Candidatura</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Estado Candidatura</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Análise da IA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notas Pessoais</t>
         </is>
@@ -740,21 +1062,21 @@
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="5" t="n">
-        <v>74</v>
+        <v>72.5</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>DATA SCIENCE CONSULTANT LISBON</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Management Solutions</t>
+          <t>Know to grow</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Lisboa, Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -769,12 +1091,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>python, machine learning, monte carlo</t>
+          <t>python</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Junior (0-1 ano)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -784,33 +1106,43 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>ITJobs.pt</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e PySpark</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>Estamos a contratar - Engenheiro(a) Informático(a) - Inteligência Artificial</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Hotel FeelViana</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -830,12 +1162,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>python, sql, pandas, numpy, git</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -845,33 +1177,43 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:29:58</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Inteligência Artificial, Machine Learning ou IA Generativa</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>The Key Talent - AI Engineer  Agent Designer</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>THE KEY TALENT PORTUGAL LDA</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -891,12 +1233,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>python, rag, llm</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Mid-Senior</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -906,38 +1248,48 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:30:00</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Vaga está relacionada com IA e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Data Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>PrimeIT</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -952,12 +1304,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>python, sql</t>
+          <t>python, pandas, numpy, langchain, embeddings, rag, llm, machine learning</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -967,33 +1319,43 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:30:09</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, conhecimentos em ML e LLM adequados</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>BI Machine Learning BI/26_016_ConvergeAI_EPMQ</t>
+          <t>Applied AI Engineer - AI Finance Agent</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>BJAK</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1013,12 +1375,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>python, fastapi, llm, machine learning</t>
+          <t>python, rag, llm</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1028,38 +1390,48 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:30:16</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, oportunidade de trabalhar em AI Finance Agent</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Estamos a contratar - Engenheiro(a) Informático(a) - Inteligência Artificial</t>
+          <t>GenAI Engineer</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Lisboa, Lisbon, Portugal</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1074,12 +1446,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>python, sql, langchain, embeddings, git, rag, llm</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1089,33 +1461,43 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:30:24</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de engenharia de GenAI adequada para recém-licenciado</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5" t="n">
-        <v>65</v>
+        <v>70.5</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Analista IA (M/F)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Palmtop - Tecnologia</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1135,12 +1517,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>python, sql, llm, machine learning</t>
+          <t>python, machine learning</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1150,33 +1532,43 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de IA, Python e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The Key Talent - AI Engineer  Agent Designer</t>
+          <t>Python engineer (registry api)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Intellias</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1186,7 +1578,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Presencial / Híbrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1196,12 +1588,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>python, sql, rag, llm</t>
+          <t>python</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1211,33 +1603,43 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Teamlyzer</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e AWS</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="n">
-        <v>65</v>
+        <v>67.5</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Explore Group</t>
+          <t>Neotalent Conclusion</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1257,53 +1659,63 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>langchain, huggingface, rag, nlp, llm, machine learning</t>
+          <t>python, sql, pandas, numpy, git</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>ITJobs.pt</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e SQL</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="n">
-        <v>65</v>
+        <v>67.5</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>PrimeIT</t>
+          <t>Know to grow</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1318,12 +1730,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>python, pandas, numpy, langchain, embeddings, rag, llm, machine learning</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1333,38 +1745,48 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:59</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>ITJobs.pt</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em data engineering e integração de dados</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5" t="n">
-        <v>65</v>
+        <v>67.5</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>BI Data Scientist</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>PrimeIT</t>
+          <t>Rumos Consulting</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1379,12 +1801,12 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>sql, git, llm</t>
+          <t>python, llm, machine learning</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1394,38 +1816,48 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:58</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Experiência profissional comprovada na automação de infraestrutura para formar, avaliar...</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="5" t="n">
-        <v>64</v>
+        <v>67.5</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer (AI Training)</t>
+          <t>Técnico IT - Implementação e Operação de IA</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Alignerr</t>
+          <t>Termas de Monfortinho</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Porto, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1440,12 +1872,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>python, llm, machine learning</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1455,38 +1887,48 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:30:02</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de IA, experiência não necessária</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="n">
-        <v>64</v>
+        <v>67.5</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer (AI Training)</t>
+          <t>AI &amp; Automation Solutions Developer</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Alignerr</t>
+          <t>Fujitsu</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Lisbon, Portugal</t>
+          <t>Lisboa, Lisbon, Portugal</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1501,12 +1943,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>python, llm, machine learning</t>
+          <t>python, git, rag, llm</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1516,38 +1958,48 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:25</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de desenvolvimento de soluções de IA e automação adequada...</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="5" t="n">
-        <v>61</v>
+        <v>67.5</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer - C++/Python</t>
+          <t>AI &amp; Automation Solutions Developer</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Fujitsu</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Greater Braga Area</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1562,12 +2014,12 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>python, sql</t>
+          <t>python, git, rag, llm</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1577,33 +2029,43 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:30:26</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M15" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de desenvolvimento de soluções de IA e automação adequada...</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="5" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Analista IA (M/F)</t>
+          <t>Engenheiro Eletrotécnico  IA, Dados e Sistemas Inteligentes (M/F) - Covilhã</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Hexawatt, Lda</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1623,12 +2085,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>python, machine learning</t>
+          <t>python, scikit-learn, machine learning</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1638,33 +2100,43 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M16" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de Engenharia Eletrotécnica com IA e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Data Analyst (4 day workweek &amp; remote)</t>
+          <t>Engenheiro Eletrotécnico  IA, Dados e Sistemas Inteligentes (M/F) - Porto</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Hexawatt, Lda</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1684,12 +2156,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>python, sql</t>
+          <t>python, scikit-learn, machine learning</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1699,38 +2171,48 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M17" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e análise de dados</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="5" t="n">
-        <v>61</v>
+        <v>60.5</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>AI First Developer</t>
+          <t>Data Analyst (4 day workweek &amp; remote)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Smartcat</t>
+          <t>360imprimir</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Lisboa, Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1745,432 +2227,70 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>python, llm</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:30:01</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Data Annotator - German (Lisbon - Onsite)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via Net-Empregos</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>machine learning</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>Net-Empregos</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Data Annotator - Russian (Lisbon - Onsite)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via Net-Empregos</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>machine learning</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Net-Empregos</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Junta-te à 1.ª rede de academias de IA e Tecnologia em Portugal - Transforma crianças e adolescentes</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via Net-Empregos</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Net-Empregos</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>AI Rubric Writer</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>micro1</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Remoto (Worldwide Remote)</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Himalayas</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Java ai enabled engineer</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>We Are META</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>Teamlyzer</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Técnico IT - Implementação e Operação de IA</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via Net-Empregos</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Net-Empregos</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Vaga está relacionada com Data Analytics</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Por Candidatar,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
+    <dataValidation sqref="M2:M18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por Candidatar,Candidatura feita,Cadidatura feita,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2182,22 +2302,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2248,20 +2370,30 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Data Extração</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Fonte</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Link de Candidatura</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Estado Candidatura</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Análise da IA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notas Pessoais</t>
         </is>
@@ -2269,7 +2401,7 @@
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>85</v>
+        <v>82.5</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -2278,7 +2410,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Neotalent Conclusion</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -2303,7 +2435,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Junior / Entry Level</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -2313,24 +2445,34 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
           <t>ITJobs.pt</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, foco em IA e tecnologia</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="n">
-        <v>74</v>
+      <c r="A3" s="2" t="n">
+        <v>79.5</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
@@ -2364,7 +2506,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Junior (0-1 ano)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -2374,33 +2516,43 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:36</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, habilidades relevantes</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="n">
-        <v>65</v>
+      <c r="A4" s="2" t="n">
+        <v>77.5</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Python Developer</t>
+          <t>BI Machine Learning BI/26_016_ConvergeAI_EPMQ</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Associação CCG - Centro de Computação Gráfica</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -2420,12 +2572,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>python, sql, pandas, numpy, git</t>
+          <t>python, fastapi, llm, machine learning</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -2435,101 +2587,121 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:29:57</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de Machine Learning e BI</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="n">
-        <v>65</v>
+      <c r="A5" s="2" t="n">
+        <v>77.5</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>BI Data Scientist</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>PrimeIT</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>Lisbon, Portugal</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Presencial / Híbrido</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Não especificado</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>sql, git, llm</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Recém-licenciado</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05 23:30:37</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Habilidades em BI e data science relevantes</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>BJAK</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>ITJobs.pt</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>65</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Data Engineer</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via ITJobs</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Presencial / Híbrido</t>
@@ -2542,12 +2714,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>python, sql</t>
+          <t>python, rag, llm</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -2557,33 +2729,43 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>ITJobs.pt</t>
+          <t>2026-08-05 23:30:15</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, oportunidade de trabalhar em AI-native systems</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>BI Machine Learning BI/26_016_ConvergeAI_EPMQ</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Know to grow</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2603,12 +2785,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>python, fastapi, llm, machine learning</t>
+          <t>python</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -2618,24 +2800,34 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>ITJobs.pt</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e PySpark</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -2644,7 +2836,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Hotel FeelViana</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -2669,7 +2861,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -2679,33 +2871,43 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:58</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Inteligência Artificial, Machine Learning ou IA Generativa</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>The Key Talent - AI Engineer  Agent Designer</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>THE KEY TALENT PORTUGAL LDA</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -2725,12 +2927,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>python, sql, llm, machine learning</t>
+          <t>python, rag, llm</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Mid-Senior</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -2740,38 +2942,48 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:00</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Vaga está relacionada com IA e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The Key Talent - AI Engineer  Agent Designer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>PrimeIT</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Lisbon, Portugal</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -2786,12 +2998,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>python, sql, rag, llm</t>
+          <t>python, pandas, numpy, langchain, embeddings, rag, llm, machine learning</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -2801,33 +3013,43 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:30:09</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, conhecimentos em ML e LLM adequados</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer</t>
+          <t>Applied AI Engineer - AI Finance Agent</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Explore Group</t>
+          <t>BJAK</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -2847,53 +3069,63 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>langchain, huggingface, rag, nlp, llm, machine learning</t>
+          <t>python, rag, llm</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:16</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Experiência não exigida, oportunidade de trabalhar em AI Finance Agent</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5" t="n">
-        <v>65</v>
+        <v>72.5</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer</t>
+          <t>GenAI Engineer</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>PrimeIT</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>Lisboa, Lisbon, Portugal</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -2908,12 +3140,12 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>python, pandas, numpy, langchain, embeddings, rag, llm, machine learning</t>
+          <t>python, sql, langchain, embeddings, git, rag, llm</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -2923,38 +3155,48 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:24</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de engenharia de GenAI adequada para recém-licenciado</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="5" t="n">
-        <v>65</v>
+        <v>70.5</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>BI Data Scientist</t>
+          <t>Analista IA (M/F)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>PrimeIT</t>
+          <t>Palmtop - Tecnologia</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2969,12 +3211,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>sql, git, llm</t>
+          <t>python, machine learning</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -2984,43 +3226,53 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:57</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de IA, Python e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer (AI Training)</t>
+          <t>Python engineer (registry api)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Alignerr</t>
+          <t>Intellias</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Porto, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Presencial / Híbrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -3030,12 +3282,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>python, llm, machine learning</t>
+          <t>python</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -3045,38 +3297,48 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Teamlyzer</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e AWS</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="5" t="n">
-        <v>64</v>
+        <v>67.5</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer (AI Training)</t>
+          <t>Python Developer</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Alignerr</t>
+          <t>Neotalent Conclusion</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Lisbon, Lisbon, Portugal</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -3091,12 +3353,12 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>python, llm, machine learning</t>
+          <t>python, sql, pandas, numpy, git</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -3106,33 +3368,43 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>2026-08-05 23:29:56</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>ITJobs.pt</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M15" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e SQL</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="5" t="n">
-        <v>61</v>
+        <v>67.5</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer - C++/Python</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Empresa via ITJobs</t>
+          <t>Know to grow</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -3157,7 +3429,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -3167,33 +3439,43 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:59</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
           <t>ITJobs.pt</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M16" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em data engineering e integração de dados</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n">
-        <v>61</v>
+        <v>67.5</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Analista IA (M/F)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Rumos Consulting</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -3213,12 +3495,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>python, machine learning</t>
+          <t>python, llm, machine learning</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -3228,33 +3510,43 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:58</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M17" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Experiência profissional comprovada na automação de infraestrutura para formar, avaliar...</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="5" t="n">
-        <v>61</v>
+        <v>67.5</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Data Analyst (4 day workweek &amp; remote)</t>
+          <t>Técnico IT - Implementação e Operação de IA</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Termas de Monfortinho</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -3274,12 +3566,12 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>python, sql</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -3289,33 +3581,43 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:02</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M18" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de IA, experiência não necessária</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="5" t="n">
-        <v>61</v>
+        <v>67.5</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>AI First Developer</t>
+          <t>AI &amp; Automation Solutions Developer</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Smartcat</t>
+          <t>Fujitsu</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -3335,53 +3637,63 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>python, llm</t>
+          <t>python, git, rag, llm</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:30:25</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M19" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de desenvolvimento de soluções de IA e automação adequada...</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="5" t="n">
-        <v>58</v>
+        <v>67.5</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Data Annotator - German (Lisbon - Onsite)</t>
+          <t>AI &amp; Automation Solutions Developer</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Fujitsu</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Greater Braga Area</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -3396,12 +3708,12 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>python, git, rag, llm</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -3411,33 +3723,43 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Net-Empregos</t>
+          <t>2026-08-05 23:30:26</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de desenvolvimento de soluções de IA e automação adequada...</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="5" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Data Annotator - Russian (Lisbon - Onsite)</t>
+          <t>Engenheiro Eletrotécnico  IA, Dados e Sistemas Inteligentes (M/F) - Covilhã</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Hexawatt, Lda</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3457,12 +3779,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>python, scikit-learn, machine learning</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -3472,33 +3794,43 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Vaga de Engenharia Eletrotécnica com IA e Machine Learning</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="5" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Junta-te à 1.ª rede de academias de IA e Tecnologia em Portugal - Transforma crianças e adolescentes</t>
+          <t>Engenheiro Eletrotécnico  IA, Dados e Sistemas Inteligentes (M/F) - Porto</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Empresa via Net-Empregos</t>
+          <t>Hexawatt, Lda</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -3518,12 +3850,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>python</t>
+          <t>python, scikit-learn, machine learning</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Recém-licenciado</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -3533,43 +3865,53 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
+          <t>2026-08-05 23:29:57</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
           <t>Net-Empregos</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Experiência em Python e análise de dados</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="5" t="n">
-        <v>55</v>
+        <v>60.5</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>AI Rubric Writer</t>
+          <t>Data Analyst (4 day workweek &amp; remote)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>micro1</t>
+          <t>360imprimir</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Remoto (Worldwide Remote)</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Presencial / Híbrido</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -3579,12 +3921,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>llm</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Nível Geral (Requer Verificação)</t>
+          <t>Júnior</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -3594,174 +3936,60 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Himalayas</t>
+          <t>2026-08-05 23:30:01</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Abrir Vaga 🔗</t>
+          <t>Net-Empregos</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Java ai enabled engineer</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>We Are META</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Teamlyzer</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Técnico IT - Implementação e Operação de IA</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Empresa via Net-Empregos</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Presencial / Híbrido</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Não especificado</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Nível Geral (Requer Verificação)</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Net-Empregos</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Abrir Vaga 🔗</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Por Candidatar</t>
-        </is>
-      </c>
-      <c r="M25" s="3" t="inlineStr"/>
+          <t>Abrir Vaga 🔗</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Por Candidatar</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Vaga está relacionada com Data Analytics</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Por Candidatar,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
+    <dataValidation sqref="M2:M23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por Candidatar,Candidatura feita,Cadidatura feita,Candidatado,Entrevista,Proposta,Rejeitado,Sem Resposta"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>